<commit_message>
Pruebas de ajuste e indices de modificación icils y pisa
</commit_message>
<xml_diff>
--- a/input/documents/batteries_icils_pisa_selfeff_comparison.xlsx
+++ b/input/documents/batteries_icils_pisa_selfeff_comparison.xlsx
@@ -20,7 +20,13 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="98" uniqueCount="81">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="142" uniqueCount="103">
+  <si>
+    <t xml:space="preserve">Competence area</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Competence</t>
+  </si>
   <si>
     <t xml:space="preserve">ICILS Code</t>
   </si>
@@ -40,6 +46,21 @@
     <t xml:space="preserve">Type of DSE</t>
   </si>
   <si>
+    <t xml:space="preserve">PISA CFA1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PISA CFA2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ICILS CFA1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Information and data literacy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.1 Navigate, search and filter data, information</t>
+  </si>
+  <si>
     <t xml:space="preserve">IS3G24C</t>
   </si>
   <si>
@@ -67,6 +88,9 @@
     <t xml:space="preserve">source_info</t>
   </si>
   <si>
+    <t xml:space="preserve">1.2 Evaluate data, information and digital content</t>
+  </si>
+  <si>
     <t xml:space="preserve">IS3G24J</t>
   </si>
   <si>
@@ -82,6 +106,9 @@
     <t xml:space="preserve">evaluate_info</t>
   </si>
   <si>
+    <t xml:space="preserve">1.3 Manage data, information and digital content</t>
+  </si>
+  <si>
     <t xml:space="preserve">IC183Q08JA</t>
   </si>
   <si>
@@ -100,6 +127,12 @@
     <t xml:space="preserve">install_app</t>
   </si>
   <si>
+    <t xml:space="preserve">2. Communication and collaboration</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2.1 Interact through digital technologies/2.2 Share info</t>
+  </si>
+  <si>
     <t xml:space="preserve">IC183Q03JA</t>
   </si>
   <si>
@@ -124,6 +157,9 @@
     <t xml:space="preserve">share_content</t>
   </si>
   <si>
+    <t xml:space="preserve">2.4 Collaborate through digital technologies</t>
+  </si>
+  <si>
     <t xml:space="preserve">IC183Q04JA</t>
   </si>
   <si>
@@ -133,6 +169,12 @@
     <t xml:space="preserve">pair_collab</t>
   </si>
   <si>
+    <t xml:space="preserve">3. Digital content creation</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3.1 Develop digital content</t>
+  </si>
+  <si>
     <t xml:space="preserve">IS3G24B</t>
   </si>
   <si>
@@ -145,6 +187,42 @@
     <t xml:space="preserve">write_text</t>
   </si>
   <si>
+    <t xml:space="preserve">3.1 Develop digital content / 3.2 Integrate content</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IS3G24F</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Create a multi-media presentation (with sound, pictures, or video)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IC183Q09JA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">create_media</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IS3G24H</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Insert an image into a document or message</t>
+  </si>
+  <si>
+    <t xml:space="preserve">insert_image</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3.2 Integrate and re-elaborate digital content</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IS3G24A</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Edit digital photographs or other graphic images</t>
+  </si>
+  <si>
+    <t xml:space="preserve">edit_image</t>
+  </si>
+  <si>
     <t xml:space="preserve">IS3G24D</t>
   </si>
   <si>
@@ -163,37 +241,7 @@
     <t xml:space="preserve">Specialized</t>
   </si>
   <si>
-    <t xml:space="preserve">IS3G24F</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Create a multi-media presentation (with sound, pictures, or video)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">IC183Q09JA</t>
-  </si>
-  <si>
-    <t xml:space="preserve">create_media</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Generalized</t>
-  </si>
-  <si>
-    <t xml:space="preserve">IS3G24H</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Insert an image into a document or message</t>
-  </si>
-  <si>
-    <t xml:space="preserve">insert_image</t>
-  </si>
-  <si>
-    <t xml:space="preserve">IS3G24A</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Edit digital photographs or other graphic images</t>
-  </si>
-  <si>
-    <t xml:space="preserve">edit_image</t>
+    <t xml:space="preserve">3.4 Programming</t>
   </si>
   <si>
     <t xml:space="preserve">IS3G24K</t>
@@ -220,6 +268,12 @@
     <t xml:space="preserve">visual_coding</t>
   </si>
   <si>
+    <t xml:space="preserve">4. Safety</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4.1 Protect devices/ 4.2 Protect personal data and privacy</t>
+  </si>
+  <si>
     <t xml:space="preserve">IS3G24E</t>
   </si>
   <si>
@@ -235,6 +289,12 @@
     <t xml:space="preserve">change_settings</t>
   </si>
   <si>
+    <t xml:space="preserve">5. Problem solving</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5.1 Solve technical problems</t>
+  </si>
+  <si>
     <t xml:space="preserve">IC183Q15JA</t>
   </si>
   <si>
@@ -244,7 +304,7 @@
     <t xml:space="preserve">identify_error</t>
   </si>
   <si>
-    <t xml:space="preserve">Specialized?</t>
+    <t xml:space="preserve">5.2 Identify needs and technological responses</t>
   </si>
   <si>
     <t xml:space="preserve">IC183Q13JA</t>
@@ -254,6 +314,12 @@
   </si>
   <si>
     <t xml:space="preserve">identify_app</t>
+  </si>
+  <si>
+    <t xml:space="preserve">|</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5.3 Use digital technologies creatively</t>
   </si>
   <si>
     <t xml:space="preserve">IC183Q16JA</t>
@@ -304,7 +370,7 @@
       <charset val="1"/>
     </font>
     <font>
-      <u val="single"/>
+      <i val="true"/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -312,7 +378,7 @@
       <charset val="1"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -321,8 +387,32 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="0"/>
+        <fgColor rgb="FFFFAA95"/>
+        <bgColor rgb="FFE6B9B8"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFAFD095"/>
+        <bgColor rgb="FFB7B3CA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFE8F2A1"/>
         <bgColor rgb="FFFFFFCC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFB7B3CA"/>
+        <bgColor rgb="FFE6B9B8"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.5999"/>
+        <bgColor rgb="FFFFAA95"/>
       </patternFill>
     </fill>
   </fills>
@@ -367,45 +457,141 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="34">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="5" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="5" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="6" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -417,6 +603,66 @@
     <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
     <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="FF000000"/>
+      <rgbColor rgb="FFFFFFFF"/>
+      <rgbColor rgb="FFFF0000"/>
+      <rgbColor rgb="FF00FF00"/>
+      <rgbColor rgb="FF0000FF"/>
+      <rgbColor rgb="FFFFFF00"/>
+      <rgbColor rgb="FFFF00FF"/>
+      <rgbColor rgb="FF00FFFF"/>
+      <rgbColor rgb="FF800000"/>
+      <rgbColor rgb="FF008000"/>
+      <rgbColor rgb="FF000080"/>
+      <rgbColor rgb="FF808000"/>
+      <rgbColor rgb="FF800080"/>
+      <rgbColor rgb="FF008080"/>
+      <rgbColor rgb="FFB7B3CA"/>
+      <rgbColor rgb="FF808080"/>
+      <rgbColor rgb="FF9999FF"/>
+      <rgbColor rgb="FF993366"/>
+      <rgbColor rgb="FFFFFFCC"/>
+      <rgbColor rgb="FFCCFFFF"/>
+      <rgbColor rgb="FF660066"/>
+      <rgbColor rgb="FFFF8080"/>
+      <rgbColor rgb="FF0066CC"/>
+      <rgbColor rgb="FFCCCCFF"/>
+      <rgbColor rgb="FF000080"/>
+      <rgbColor rgb="FFFF00FF"/>
+      <rgbColor rgb="FFFFFF00"/>
+      <rgbColor rgb="FF00FFFF"/>
+      <rgbColor rgb="FF800080"/>
+      <rgbColor rgb="FF800000"/>
+      <rgbColor rgb="FF008080"/>
+      <rgbColor rgb="FF0000FF"/>
+      <rgbColor rgb="FF00CCFF"/>
+      <rgbColor rgb="FFCCFFFF"/>
+      <rgbColor rgb="FFCCFFCC"/>
+      <rgbColor rgb="FFE8F2A1"/>
+      <rgbColor rgb="FFAFD095"/>
+      <rgbColor rgb="FFFFAA95"/>
+      <rgbColor rgb="FFCC99FF"/>
+      <rgbColor rgb="FFE6B9B8"/>
+      <rgbColor rgb="FF3366FF"/>
+      <rgbColor rgb="FF33CCCC"/>
+      <rgbColor rgb="FF99CC00"/>
+      <rgbColor rgb="FFFFCC00"/>
+      <rgbColor rgb="FFFF9900"/>
+      <rgbColor rgb="FFFF6600"/>
+      <rgbColor rgb="FF666699"/>
+      <rgbColor rgb="FF969696"/>
+      <rgbColor rgb="FF003366"/>
+      <rgbColor rgb="FF339966"/>
+      <rgbColor rgb="FF003300"/>
+      <rgbColor rgb="FF333300"/>
+      <rgbColor rgb="FF993300"/>
+      <rgbColor rgb="FF993366"/>
+      <rgbColor rgb="FF333399"/>
+      <rgbColor rgb="FF333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
@@ -600,403 +846,770 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:T20"/>
+  <dimension ref="A1:R1048576"/>
   <sheetFormatPr defaultColWidth="8.59765625" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="13"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="54.37"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="16.18"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="54.18"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="26.91"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="18.82"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16384" min="16373" style="0" width="10.16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="32.36"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="2" width="47.37"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="2" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="2" width="54.37"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="2" width="16.18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="2" width="54.18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="26.91"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="18.82"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="14.82"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="21"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="14.18"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="2" t="s">
+      <c r="B1" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="D1" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="E1" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="F1" s="4" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="2" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="3" t="s">
+      <c r="G1" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="H1" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="I1" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="D2" s="3" t="s">
+      <c r="J1" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="E2" s="4" t="s">
+      <c r="K1" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="F2" s="5" t="s">
+    </row>
+    <row r="2" s="9" customFormat="true" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="6" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="3" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="3" t="s">
+      <c r="B2" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="C2" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="C3" s="3"/>
-      <c r="D3" s="3"/>
-      <c r="E3" s="4" t="s">
+      <c r="D2" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="F3" s="5" t="s">
+      <c r="E2" s="7" t="s">
+        <v>15</v>
+      </c>
+      <c r="F2" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="G2" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="H2" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="I2" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="K2" s="8" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" s="9" customFormat="true" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="6" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="4" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="B4" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="C4" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="D4" s="3" t="s">
+      <c r="B3" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="C3" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="D3" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="E3" s="7"/>
+      <c r="F3" s="7"/>
+      <c r="G3" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="H3" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="E4" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="F4" s="5" t="s">
+      <c r="I3" s="8"/>
+      <c r="J3" s="8"/>
+      <c r="K3" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="O3" s="10"/>
+      <c r="P3" s="10"/>
+      <c r="Q3" s="10"/>
+      <c r="R3" s="10"/>
+    </row>
+    <row r="4" s="9" customFormat="true" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="6" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="5" s="7" customFormat="true" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="4"/>
-      <c r="B5" s="6"/>
-      <c r="C5" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="D5" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="E5" s="4" t="s">
+      <c r="B4" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="F5" s="6" t="s">
+      <c r="C4" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="D4" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="E4" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="F4" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="G4" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="H4" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="I4" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="J4" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="K4" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="O4" s="10"/>
+      <c r="P4" s="10"/>
+      <c r="Q4" s="10"/>
+      <c r="R4" s="10"/>
+    </row>
+    <row r="5" s="9" customFormat="true" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="G5" s="0"/>
-      <c r="H5" s="0"/>
-      <c r="I5" s="0"/>
-      <c r="J5" s="0"/>
-      <c r="K5" s="0"/>
-      <c r="L5" s="0"/>
-      <c r="M5" s="0"/>
-      <c r="N5" s="0"/>
-      <c r="O5" s="0"/>
-      <c r="P5" s="0"/>
-      <c r="Q5" s="0"/>
-      <c r="R5" s="0"/>
-      <c r="S5" s="0"/>
-      <c r="T5" s="0"/>
-    </row>
-    <row r="6" s="7" customFormat="true" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="4" t="s">
-        <v>23</v>
-      </c>
-      <c r="B6" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="C6" s="4"/>
-      <c r="D6" s="4"/>
-      <c r="E6" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="F6" s="6" t="s">
+      <c r="B5" s="7" t="s">
+        <v>28</v>
+      </c>
+      <c r="C5" s="7"/>
+      <c r="D5" s="8"/>
+      <c r="E5" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="F5" s="7" t="s">
+        <v>30</v>
+      </c>
+      <c r="G5" s="7" t="s">
+        <v>31</v>
+      </c>
+      <c r="H5" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="I5" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="J5" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="K5" s="8"/>
+      <c r="O5" s="10"/>
+      <c r="P5" s="10"/>
+      <c r="Q5" s="10"/>
+      <c r="R5" s="10"/>
+    </row>
+    <row r="6" s="9" customFormat="true" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="G6" s="0"/>
-      <c r="H6" s="0"/>
-      <c r="I6" s="0"/>
-      <c r="J6" s="0"/>
-      <c r="K6" s="0"/>
-      <c r="L6" s="0"/>
-      <c r="M6" s="0"/>
-      <c r="N6" s="0"/>
-      <c r="O6" s="0"/>
-      <c r="P6" s="0"/>
-      <c r="Q6" s="0"/>
-      <c r="R6" s="0"/>
-      <c r="S6" s="0"/>
-      <c r="T6" s="0"/>
-    </row>
-    <row r="7" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="3"/>
-      <c r="B7" s="3"/>
-      <c r="C7" s="3" t="s">
-        <v>26</v>
-      </c>
-      <c r="D7" s="3" t="s">
-        <v>27</v>
-      </c>
-      <c r="E7" s="4" t="s">
+      <c r="B6" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="F7" s="5" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="B8" s="3" t="s">
-        <v>30</v>
-      </c>
-      <c r="C8" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="D8" s="3" t="s">
+      <c r="C6" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="E8" s="4" t="s">
+      <c r="D6" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="F8" s="5" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="3"/>
-      <c r="B9" s="3"/>
-      <c r="C9" s="3" t="s">
+      <c r="E6" s="7"/>
+      <c r="F6" s="7"/>
+      <c r="G6" s="7" t="s">
         <v>34</v>
       </c>
-      <c r="D9" s="3" t="s">
+      <c r="H6" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="I6" s="8"/>
+      <c r="J6" s="8"/>
+      <c r="K6" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="O6" s="10"/>
+      <c r="P6" s="10"/>
+      <c r="Q6" s="10"/>
+      <c r="R6" s="10"/>
+    </row>
+    <row r="7" s="14" customFormat="true" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="11" t="s">
         <v>35</v>
       </c>
-      <c r="E9" s="4" t="s">
+      <c r="B7" s="12" t="s">
         <v>36</v>
       </c>
-      <c r="F9" s="5" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="3" t="s">
+      <c r="C7" s="11"/>
+      <c r="D7" s="11"/>
+      <c r="E7" s="11" t="s">
         <v>37</v>
       </c>
-      <c r="B10" s="3" t="s">
+      <c r="F7" s="11" t="s">
         <v>38</v>
       </c>
-      <c r="C10" s="3" t="s">
+      <c r="G7" s="11" t="s">
         <v>39</v>
       </c>
-      <c r="D10" s="3" t="s">
-        <v>38</v>
-      </c>
-      <c r="E10" s="4" t="s">
+      <c r="H7" s="13" t="s">
+        <v>18</v>
+      </c>
+      <c r="I7" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="J7" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="K7" s="13"/>
+      <c r="O7" s="15"/>
+      <c r="P7" s="15"/>
+      <c r="Q7" s="15"/>
+      <c r="R7" s="15"/>
+    </row>
+    <row r="8" s="14" customFormat="true" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="12" t="s">
+        <v>35</v>
+      </c>
+      <c r="B8" s="12" t="s">
+        <v>36</v>
+      </c>
+      <c r="C8" s="11" t="s">
         <v>40</v>
       </c>
-      <c r="F10" s="5" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="38.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="3" t="s">
+      <c r="D8" s="11" t="s">
         <v>41</v>
       </c>
-      <c r="B11" s="3" t="s">
+      <c r="E8" s="11" t="s">
         <v>42</v>
       </c>
-      <c r="C11" s="3" t="s">
+      <c r="F8" s="11" t="s">
         <v>43</v>
       </c>
-      <c r="D11" s="3" t="s">
+      <c r="G8" s="11" t="s">
         <v>44</v>
       </c>
-      <c r="E11" s="4" t="s">
+      <c r="H8" s="13" t="s">
+        <v>18</v>
+      </c>
+      <c r="I8" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="J8" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="K8" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="O8" s="16"/>
+      <c r="P8" s="16"/>
+      <c r="Q8" s="16"/>
+      <c r="R8" s="16"/>
+    </row>
+    <row r="9" s="14" customFormat="true" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="11" t="s">
+        <v>35</v>
+      </c>
+      <c r="B9" s="11" t="s">
         <v>45</v>
       </c>
-      <c r="F11" s="5" t="s">
+      <c r="C9" s="11"/>
+      <c r="D9" s="11"/>
+      <c r="E9" s="11" t="s">
         <v>46</v>
       </c>
-    </row>
-    <row r="12" customFormat="false" ht="40.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="3" t="s">
+      <c r="F9" s="11" t="s">
         <v>47</v>
       </c>
-      <c r="B12" s="3" t="s">
+      <c r="G9" s="11" t="s">
         <v>48</v>
       </c>
-      <c r="C12" s="3" t="s">
+      <c r="H9" s="13" t="s">
+        <v>18</v>
+      </c>
+      <c r="I9" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="J9" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="K9" s="13"/>
+      <c r="O9" s="15"/>
+      <c r="P9" s="15"/>
+      <c r="Q9" s="15"/>
+      <c r="R9" s="15"/>
+    </row>
+    <row r="10" s="20" customFormat="true" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="17" t="s">
         <v>49</v>
       </c>
-      <c r="D12" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="E12" s="4" t="s">
+      <c r="B10" s="17" t="s">
         <v>50</v>
       </c>
-      <c r="F12" s="5" t="s">
+      <c r="C10" s="18" t="s">
         <v>51</v>
       </c>
-    </row>
-    <row r="13" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="3" t="s">
+      <c r="D10" s="18" t="s">
         <v>52</v>
       </c>
-      <c r="B13" s="3" t="s">
+      <c r="E10" s="18" t="s">
         <v>53</v>
       </c>
-      <c r="C13" s="3"/>
-      <c r="D13" s="3"/>
-      <c r="E13" s="3" t="s">
+      <c r="F10" s="18" t="s">
+        <v>52</v>
+      </c>
+      <c r="G10" s="18" t="s">
         <v>54</v>
       </c>
-      <c r="F13" s="5" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="14" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="3" t="s">
+      <c r="H10" s="19" t="s">
+        <v>18</v>
+      </c>
+      <c r="I10" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="J10" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="K10" s="19" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11" s="20" customFormat="true" ht="40.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="17" t="s">
+        <v>49</v>
+      </c>
+      <c r="B11" s="17" t="s">
         <v>55</v>
       </c>
-      <c r="B14" s="3" t="s">
+      <c r="C11" s="18" t="s">
         <v>56</v>
       </c>
-      <c r="C14" s="3"/>
-      <c r="D14" s="3"/>
-      <c r="E14" s="3" t="s">
+      <c r="D11" s="18" t="s">
         <v>57</v>
       </c>
-      <c r="F14" s="5" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="15" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="3" t="s">
+      <c r="E11" s="18" t="s">
         <v>58</v>
       </c>
-      <c r="B15" s="3" t="s">
+      <c r="F11" s="18" t="s">
+        <v>57</v>
+      </c>
+      <c r="G11" s="18" t="s">
         <v>59</v>
       </c>
-      <c r="C15" s="3" t="s">
+      <c r="H11" s="19" t="s">
+        <v>18</v>
+      </c>
+      <c r="I11" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="J11" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="K11" s="19" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" s="20" customFormat="true" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="17" t="s">
+        <v>49</v>
+      </c>
+      <c r="B12" s="17" t="s">
+        <v>55</v>
+      </c>
+      <c r="C12" s="18" t="s">
         <v>60</v>
       </c>
-      <c r="D15" s="3" t="s">
+      <c r="D12" s="18" t="s">
         <v>61</v>
       </c>
-      <c r="E15" s="3" t="s">
+      <c r="E12" s="18"/>
+      <c r="F12" s="18"/>
+      <c r="G12" s="18" t="s">
         <v>62</v>
       </c>
-      <c r="F15" s="5" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="16" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="3" t="s">
+      <c r="H12" s="19" t="s">
+        <v>18</v>
+      </c>
+      <c r="I12" s="19"/>
+      <c r="J12" s="19"/>
+      <c r="K12" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="O12" s="21"/>
+      <c r="P12" s="21"/>
+      <c r="Q12" s="21"/>
+      <c r="R12" s="21"/>
+    </row>
+    <row r="13" s="20" customFormat="true" ht="16.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="17" t="s">
+        <v>49</v>
+      </c>
+      <c r="B13" s="17" t="s">
         <v>63</v>
       </c>
-      <c r="B16" s="3" t="s">
+      <c r="C13" s="18" t="s">
         <v>64</v>
       </c>
-      <c r="C16" s="3"/>
-      <c r="D16" s="3"/>
-      <c r="E16" s="3" t="s">
+      <c r="D13" s="18" t="s">
         <v>65</v>
       </c>
-      <c r="F16" s="5" t="s">
-        <v>46</v>
-      </c>
+      <c r="E13" s="18"/>
+      <c r="F13" s="18"/>
+      <c r="G13" s="18" t="s">
+        <v>66</v>
+      </c>
+      <c r="H13" s="19" t="s">
+        <v>18</v>
+      </c>
+      <c r="I13" s="19"/>
+      <c r="J13" s="19"/>
+      <c r="K13" s="19" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14" s="25" customFormat="true" ht="38.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="22" t="s">
+        <v>49</v>
+      </c>
+      <c r="B14" s="22" t="s">
+        <v>50</v>
+      </c>
+      <c r="C14" s="23" t="s">
+        <v>67</v>
+      </c>
+      <c r="D14" s="23" t="s">
+        <v>68</v>
+      </c>
+      <c r="E14" s="23" t="s">
+        <v>69</v>
+      </c>
+      <c r="F14" s="23" t="s">
+        <v>70</v>
+      </c>
+      <c r="G14" s="23" t="s">
+        <v>71</v>
+      </c>
+      <c r="H14" s="24" t="s">
+        <v>72</v>
+      </c>
+      <c r="I14" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="J14" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="K14" s="24" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15" s="25" customFormat="true" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="22" t="s">
+        <v>49</v>
+      </c>
+      <c r="B15" s="22" t="s">
+        <v>73</v>
+      </c>
+      <c r="C15" s="23" t="s">
+        <v>74</v>
+      </c>
+      <c r="D15" s="23" t="s">
+        <v>75</v>
+      </c>
+      <c r="E15" s="23" t="s">
+        <v>76</v>
+      </c>
+      <c r="F15" s="23" t="s">
+        <v>77</v>
+      </c>
+      <c r="G15" s="23" t="s">
+        <v>78</v>
+      </c>
+      <c r="H15" s="24" t="s">
+        <v>72</v>
+      </c>
+      <c r="I15" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="J15" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="K15" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="O15" s="26"/>
+      <c r="P15" s="26"/>
+      <c r="Q15" s="26"/>
+      <c r="R15" s="26"/>
+    </row>
+    <row r="16" s="25" customFormat="true" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="22" t="s">
+        <v>49</v>
+      </c>
+      <c r="B16" s="22" t="s">
+        <v>73</v>
+      </c>
+      <c r="C16" s="23" t="s">
+        <v>79</v>
+      </c>
+      <c r="D16" s="23" t="s">
+        <v>80</v>
+      </c>
+      <c r="E16" s="23"/>
+      <c r="F16" s="23"/>
+      <c r="G16" s="23" t="s">
+        <v>81</v>
+      </c>
+      <c r="H16" s="24" t="s">
+        <v>72</v>
+      </c>
+      <c r="I16" s="24"/>
+      <c r="J16" s="24"/>
+      <c r="K16" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="O16" s="26"/>
+      <c r="P16" s="26"/>
+      <c r="Q16" s="26"/>
+      <c r="R16" s="26"/>
     </row>
     <row r="17" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="3" t="s">
-        <v>66</v>
-      </c>
-      <c r="B17" s="3" t="s">
-        <v>67</v>
-      </c>
-      <c r="C17" s="3" t="s">
-        <v>68</v>
-      </c>
-      <c r="D17" s="3" t="s">
-        <v>69</v>
-      </c>
-      <c r="E17" s="3" t="s">
-        <v>70</v>
-      </c>
-      <c r="F17" s="5" t="s">
-        <v>11</v>
-      </c>
+      <c r="A17" s="27" t="s">
+        <v>82</v>
+      </c>
+      <c r="B17" s="28" t="s">
+        <v>83</v>
+      </c>
+      <c r="C17" s="27" t="s">
+        <v>84</v>
+      </c>
+      <c r="D17" s="27" t="s">
+        <v>85</v>
+      </c>
+      <c r="E17" s="27" t="s">
+        <v>86</v>
+      </c>
+      <c r="F17" s="27" t="s">
+        <v>87</v>
+      </c>
+      <c r="G17" s="27" t="s">
+        <v>88</v>
+      </c>
+      <c r="H17" s="29" t="s">
+        <v>18</v>
+      </c>
+      <c r="I17" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="J17" s="29" t="n">
+        <v>1</v>
+      </c>
+      <c r="K17" s="29" t="n">
+        <v>1</v>
+      </c>
+      <c r="O17" s="30"/>
+      <c r="P17" s="30"/>
+      <c r="Q17" s="30"/>
+      <c r="R17" s="30"/>
     </row>
     <row r="18" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="8"/>
-      <c r="B18" s="8"/>
-      <c r="C18" s="8" t="s">
-        <v>71</v>
-      </c>
-      <c r="D18" s="8" t="s">
+      <c r="A18" s="31" t="s">
+        <v>89</v>
+      </c>
+      <c r="B18" s="31" t="s">
+        <v>90</v>
+      </c>
+      <c r="C18" s="32"/>
+      <c r="D18" s="32"/>
+      <c r="E18" s="32" t="s">
+        <v>91</v>
+      </c>
+      <c r="F18" s="32" t="s">
+        <v>92</v>
+      </c>
+      <c r="G18" s="32" t="s">
+        <v>93</v>
+      </c>
+      <c r="H18" s="29" t="s">
         <v>72</v>
       </c>
-      <c r="E18" s="8" t="s">
-        <v>73</v>
-      </c>
-      <c r="F18" s="5" t="s">
-        <v>74</v>
-      </c>
+      <c r="I18" s="29" t="n">
+        <v>1</v>
+      </c>
+      <c r="J18" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="K18" s="29"/>
+      <c r="O18" s="30"/>
+      <c r="P18" s="30"/>
+      <c r="Q18" s="30"/>
+      <c r="R18" s="30"/>
     </row>
     <row r="19" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="8"/>
-      <c r="B19" s="8"/>
-      <c r="C19" s="8" t="s">
-        <v>75</v>
-      </c>
-      <c r="D19" s="8" t="s">
-        <v>76</v>
-      </c>
-      <c r="E19" s="8" t="s">
-        <v>77</v>
-      </c>
-      <c r="F19" s="5" t="s">
-        <v>74</v>
-      </c>
+      <c r="A19" s="31" t="s">
+        <v>89</v>
+      </c>
+      <c r="B19" s="31" t="s">
+        <v>94</v>
+      </c>
+      <c r="C19" s="32"/>
+      <c r="D19" s="32"/>
+      <c r="E19" s="32" t="s">
+        <v>95</v>
+      </c>
+      <c r="F19" s="32" t="s">
+        <v>96</v>
+      </c>
+      <c r="G19" s="32" t="s">
+        <v>97</v>
+      </c>
+      <c r="H19" s="29" t="s">
+        <v>72</v>
+      </c>
+      <c r="I19" s="29" t="s">
+        <v>98</v>
+      </c>
+      <c r="J19" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="K19" s="29"/>
+      <c r="O19" s="30"/>
+      <c r="P19" s="30"/>
+      <c r="Q19" s="30"/>
+      <c r="R19" s="30"/>
     </row>
     <row r="20" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="8"/>
-      <c r="B20" s="8"/>
-      <c r="C20" s="8" t="s">
-        <v>78</v>
-      </c>
-      <c r="D20" s="8" t="s">
-        <v>79</v>
-      </c>
-      <c r="E20" s="8" t="s">
-        <v>80</v>
-      </c>
-      <c r="F20" s="5" t="s">
-        <v>74</v>
-      </c>
-      <c r="G20" s="9"/>
-    </row>
+      <c r="A20" s="31" t="s">
+        <v>89</v>
+      </c>
+      <c r="B20" s="31" t="s">
+        <v>99</v>
+      </c>
+      <c r="C20" s="32"/>
+      <c r="D20" s="32"/>
+      <c r="E20" s="32" t="s">
+        <v>100</v>
+      </c>
+      <c r="F20" s="32" t="s">
+        <v>101</v>
+      </c>
+      <c r="G20" s="32" t="s">
+        <v>102</v>
+      </c>
+      <c r="H20" s="29" t="s">
+        <v>72</v>
+      </c>
+      <c r="I20" s="29" t="n">
+        <v>1</v>
+      </c>
+      <c r="J20" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="K20" s="29"/>
+      <c r="O20" s="30"/>
+      <c r="P20" s="30"/>
+      <c r="Q20" s="30"/>
+      <c r="R20" s="33"/>
+    </row>
+    <row r="21" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="O21" s="30"/>
+      <c r="P21" s="30"/>
+      <c r="Q21" s="30"/>
+      <c r="R21" s="33"/>
+    </row>
+    <row r="22" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="O22" s="30"/>
+      <c r="P22" s="30"/>
+      <c r="Q22" s="30"/>
+      <c r="R22" s="33"/>
+    </row>
+    <row r="23" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="O23" s="30"/>
+      <c r="P23" s="30"/>
+      <c r="Q23" s="30"/>
+      <c r="R23" s="33"/>
+    </row>
+    <row r="24" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="O24" s="30"/>
+      <c r="P24" s="30"/>
+      <c r="Q24" s="30"/>
+      <c r="R24" s="33"/>
+    </row>
+    <row r="25" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="O25" s="30"/>
+      <c r="P25" s="30"/>
+      <c r="Q25" s="30"/>
+      <c r="R25" s="33"/>
+    </row>
+    <row r="26" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="O26" s="30"/>
+      <c r="P26" s="30"/>
+      <c r="Q26" s="30"/>
+      <c r="R26" s="33"/>
+    </row>
+    <row r="27" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="O27" s="30"/>
+      <c r="P27" s="30"/>
+      <c r="Q27" s="30"/>
+      <c r="R27" s="33"/>
+    </row>
+    <row r="28" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="O28" s="30"/>
+      <c r="P28" s="30"/>
+      <c r="Q28" s="30"/>
+      <c r="R28" s="33"/>
+    </row>
+    <row r="29" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="O29" s="30"/>
+      <c r="P29" s="30"/>
+      <c r="Q29" s="30"/>
+      <c r="R29" s="33"/>
+    </row>
+    <row r="30" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="O30" s="30"/>
+      <c r="P30" s="30"/>
+      <c r="Q30" s="30"/>
+      <c r="R30" s="33"/>
+    </row>
+    <row r="31" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="O31" s="30"/>
+      <c r="P31" s="30"/>
+      <c r="Q31" s="30"/>
+      <c r="R31" s="33"/>
+    </row>
+    <row r="1048575" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>